<commit_message>
adr-007 added, update to adr-002
</commit_message>
<xml_diff>
--- a/docs/discovery/Design Playbook - Quack.xlsx
+++ b/docs/discovery/Design Playbook - Quack.xlsx
@@ -6895,11 +6895,31 @@
       </c>
     </row>
     <row r="10" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="2"/>
-      <c r="B10" s="2"/>
-      <c r="C10" s="2"/>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>DL-07</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Repository and stack layout</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Monorepo; one CDK stack per deployable; one ECS service per HTTP domain; no CloudFormation exports</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>docs/adr/adr-007-stack-layout.md</t>
+        </is>
+      </c>
     </row>
     <row r="11" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2"/>

</xml_diff>

<commit_message>
added adr-008 and draft architecture.md
</commit_message>
<xml_diff>
--- a/docs/discovery/Design Playbook - Quack.xlsx
+++ b/docs/discovery/Design Playbook - Quack.xlsx
@@ -6922,11 +6922,31 @@
       </c>
     </row>
     <row r="11" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="2"/>
-      <c r="B11" s="2"/>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>DL-08</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Cross-domain reads</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Direct read of another domain's records under a stated rule; no service-to-service calls in the MVP</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>docs/adr/adr-008-cross-domain-reads.md</t>
+        </is>
+      </c>
     </row>
     <row r="12" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2"/>

</xml_diff>

<commit_message>
updated architecture, renamed tenants to ponds
</commit_message>
<xml_diff>
--- a/docs/discovery/Design Playbook - Quack.xlsx
+++ b/docs/discovery/Design Playbook - Quack.xlsx
@@ -487,7 +487,7 @@
     <t>Does access need role based access control (RBAC), record level access, or both?</t>
   </si>
   <si>
-    <t>Is this multi tenant, and how strict must tenant isolation be?</t>
+    <t>Is this multi pond, and how strict must pond isolation be?</t>
   </si>
   <si>
     <t>What must be auditable, and who consumes the audit trail?</t>
@@ -1238,10 +1238,10 @@
     <t>OOS-09</t>
   </si>
   <si>
-    <t>Multi-tenancy</t>
-  </si>
-  <si>
-    <t>Single tenant required; tenant key kept in the data model</t>
+    <t>Multiple ponds</t>
+  </si>
+  <si>
+    <t>Single pond required; pond key kept in the data model</t>
   </si>
   <si>
     <t>Named future enhancement</t>
@@ -1421,7 +1421,7 @@
     <t>OOS-11</t>
   </si>
   <si>
-    <t>No compliance program (GDPR, CCPA, SOC 2); owner and member roles only, no admin role; request logs only, no exportable audit log. Tenancy is OOS-09.</t>
+    <t>No compliance program (GDPR, CCPA, SOC 2); owner and member roles only, no admin role; request logs only, no exportable audit log. Ponds are OOS-09.</t>
   </si>
   <si>
     <t>GDPR and CCPA; SOC 2 Type II as the control framework. Privacy Operations owner TBD*</t>
@@ -1433,10 +1433,10 @@
     <t>Record level. Flock membership for read and write; ownership for delete.</t>
   </si>
   <si>
-    <t>Multi-tenant with strict isolation: every query scoped by tenant.*</t>
-  </si>
-  <si>
-    <t>Single tenant in demo, but with data model shaped to include tenancy. See OOS-09.</t>
+    <t>Multi-pond with strict isolation: every query scoped by pond.*</t>
+  </si>
+  <si>
+    <t>Single pond in demo, but with data model shaped to include ponds. See OOS-09.</t>
   </si>
   <si>
     <t xml:space="preserve">Sign-ins, flock create and delete, and member additions. Non-deleted message history only. Compliance officers TBD. </t>
@@ -1622,10 +1622,10 @@
     <t>NFR-11</t>
   </si>
   <si>
-    <t>Record-level tenant isolation</t>
-  </si>
-  <si>
-    <t>Every record carries the tenant key. One hardcoded tenant is used.</t>
+    <t>Record-level pond isolation</t>
+  </si>
+  <si>
+    <t>Every record carries the pond key. One hardcoded pond is used.</t>
   </si>
   <si>
     <t>OOS-09; FC-01</t>
@@ -1634,10 +1634,10 @@
     <t>12 to 24 months</t>
   </si>
   <si>
-    <t>Key rewrite and data migration if the tenant key is absent from any key</t>
-  </si>
-  <si>
-    <t>Tenant key in every key now; nothing else built</t>
+    <t>Key rewrite and data migration if the pond key is absent from any key</t>
+  </si>
+  <si>
+    <t>Pond key in every key now; nothing else built</t>
   </si>
   <si>
     <t>FC-02</t>
@@ -1709,7 +1709,7 @@
     <t>A person who has signed in</t>
   </si>
   <si>
-    <t>tenantId, duckId, googleSubject, email, displayName, createdAt</t>
+    <t>pondId, duckId, googleSubject, email, displayName, createdAt</t>
   </si>
   <si>
     <t>Identity copied from the Google ID token at sign-in</t>
@@ -1724,7 +1724,7 @@
     <t>A named channel</t>
   </si>
   <si>
-    <t>tenantId, flockId, name, ownerId, createdAt</t>
+    <t>pondId, flockId, name, ownerId, createdAt</t>
   </si>
   <si>
     <t>ownerId is the creator; ownership is not transferable</t>
@@ -1739,7 +1739,7 @@
     <t>A user belongs to a flock</t>
   </si>
   <si>
-    <t>tenantId, flockId, duckId, addedBy, addedAt</t>
+    <t>pondId, flockId, duckId, addedBy, addedAt</t>
   </si>
   <si>
     <t>DE-04</t>
@@ -1751,7 +1751,7 @@
     <t>One text message in a flock</t>
   </si>
   <si>
-    <t>tenantId, flockId, messageId (time ordered), senderId (duckId), text, createdAt</t>
+    <t>pondId, flockId, messageId (time ordered), senderId (duckId), text, createdAt</t>
   </si>
   <si>
     <t>text at most 4,000 characters (ASM-03); item stays under the 400 KB limit (NFR-10)</t>
@@ -1766,7 +1766,7 @@
     <t>A live session for one user</t>
   </si>
   <si>
-    <t>tenantId, connectionId, duckId, createdAt</t>
+    <t>pondId, connectionId, duckId, createdAt</t>
   </si>
   <si>
     <t>Data Access Patterns</t>

</xml_diff>

<commit_message>
decided on data store and updated decisions
</commit_message>
<xml_diff>
--- a/docs/discovery/Design Playbook - Quack.xlsx
+++ b/docs/discovery/Design Playbook - Quack.xlsx
@@ -20,7 +20,7 @@
     <sheet name="Scale and Estimates" sheetId="4" r:id="rId5"/>
     <sheet name="Decision Log" sheetId="5" r:id="rId6"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="852" uniqueCount="675">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="858" uniqueCount="681">
   <si>
     <t>Date Created</t>
   </si>
@@ -1613,10 +1613,10 @@
     <t>Platform standard</t>
   </si>
   <si>
-    <t>A message item stays under the 400 KB item limit</t>
-  </si>
-  <si>
-    <t>https://docs.aws.amazon.com/amazondynamodb/latest/developerguide/Constraints.html</t>
+    <t>A message record stays under 400 KB</t>
+  </si>
+  <si>
+    <t>Service target. The data store ADR confirms the chosen store's record limit meets it.</t>
   </si>
   <si>
     <t>NFR-11</t>
@@ -1697,7 +1697,7 @@
     <t>If the demo outlives one month or the RPO must hold for code and operator error</t>
   </si>
   <si>
-    <t>DynamoDB Streams to a durable sink such as S3 through Firehose; after a restore, replay the gap. Keep the write path behind one module so the stream can be added without touching handlers. https://docs.aws.amazon.com/amazondynamodb/latest/developerguide/PointInTimeRecovery_Howitworks.html</t>
+    <t>A change stream from the data store to a durable sink such as S3; after a restore, replay the gap. Keep the write path behind one module so the stream can be added without touching handlers.</t>
   </si>
   <si>
     <t>Data Entities</t>
@@ -1754,7 +1754,7 @@
     <t>pondId, flockId, messageId (time ordered), senderId (duckId), text, createdAt</t>
   </si>
   <si>
-    <t>text at most 4,000 characters (ASM-03); item stays under the 400 KB limit (NFR-10)</t>
+    <t>text at most 4,000 characters (ASM-03); record stays under 400 KB (NFR-10)</t>
   </si>
   <si>
     <t>DE-05</t>
@@ -1880,10 +1880,10 @@
     <t>Put on connect; delete on disconnect</t>
   </si>
   <si>
-    <t>1,700 per second at steady state</t>
-  </si>
-  <si>
-    <t>12,000,000 users divided by the 7,200 second connection cap; higher at start of day. https://docs.aws.amazon.com/apigateway/latest/developerguide/apigateway-execution-service-websocket-limits-table.html</t>
+    <t>2,500 per second at peak</t>
+  </si>
+  <si>
+    <t>A socket lives one ID token lifetime, then the client reconnects (Assumption: 1 hour; sourced in the sign-in design). Daily active users x 9 connected hours / 1 hour / 86,400 seconds is 1,250 per second average; x2 peak ratio. Higher at start of day.</t>
   </si>
   <si>
     <t>AP-15</t>
@@ -1955,7 +1955,7 @@
     <t>Assumption: message text plus keys and attributes.</t>
   </si>
   <si>
-    <t>Assumption: table plus point-in-time recovery copy. Replicas across availability zones are not billed separately (https://aws.amazon.com/dynamodb/pricing/on-demand/).</t>
+    <t>Assumption: primary plus one backup copy</t>
   </si>
   <si>
     <t>Assumption: only recent messages are read. Entered as a fraction because the formula multiplies directly.</t>
@@ -2070,6 +2070,24 @@
   </si>
   <si>
     <t xml:space="preserve">*See OOS-10 caveat on point-in-time recovery. </t>
+  </si>
+  <si>
+    <t>Not stored. Sockets live in websocket task memory; live delivery goes through the per-flock fan-out topic (ADR-005). See AP-14 and AP-15.</t>
+  </si>
+  <si>
+    <t>Connect; disconnect (held in task memory)</t>
+  </si>
+  <si>
+    <t>Not a data store access pattern; sizes the websocket service. A socket lives one ID token lifetime, then the client reconnects (Assumption: 1 hour; sourced in the sign-in design). Daily active users x 9 connected hours / 1 hour / 86,400 seconds is 1,250 per second average; x2 peak ratio. Higher at start of day.</t>
+  </si>
+  <si>
+    <t>Find the connections of a flock's members</t>
+  </si>
+  <si>
+    <t>Not a data store access pattern. One publish per send to the flock's fan-out topic; each subscribed task pushes to its own sockets (ADR-005).</t>
+  </si>
+  <si>
+    <t>Assumption: membership check plus one put. Fan-out uses the pub/sub topic, not a data store lookup (ADR-005).</t>
   </si>
 </sst>
 </file>
@@ -5542,7 +5560,9 @@
       <c r="D8" s="2" t="s">
         <v>573</v>
       </c>
-      <c r="E8" s="2"/>
+      <c r="E8" s="2" t="s">
+        <v>675</v>
+      </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="2"/>
@@ -5892,13 +5912,13 @@
         <v>570</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>610</v>
+        <v>676</v>
       </c>
       <c r="D38" s="2" t="s">
         <v>611</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>612</v>
+        <v>677</v>
       </c>
     </row>
     <row r="39" spans="1:5" ht="28.5" x14ac:dyDescent="0.25">
@@ -5909,13 +5929,13 @@
         <v>570</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>614</v>
+        <v>678</v>
       </c>
       <c r="D39" s="2" t="s">
         <v>670</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>615</v>
+        <v>679</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
@@ -6100,13 +6120,13 @@
         <v>200</v>
       </c>
       <c r="C10" s="19">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>198</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>629</v>
+        <v>680</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="28.5" x14ac:dyDescent="0.25">
@@ -6518,7 +6538,7 @@
       </c>
       <c r="C39" s="21">
         <f>IF(COUNT($C$37,$C$10)&lt;2,"Missing Info",$C$37*$C$10)</f>
-        <v>11666.666666666666</v>
+        <v>7777.7777777777774</v>
       </c>
       <c r="D39" s="2" t="s">
         <v>249</v>

</xml_diff>

<commit_message>
finished data model design
</commit_message>
<xml_diff>
--- a/docs/discovery/Design Playbook - Quack.xlsx
+++ b/docs/discovery/Design Playbook - Quack.xlsx
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="858" uniqueCount="681">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="862" uniqueCount="685">
   <si>
     <t>Date Created</t>
   </si>
@@ -2088,6 +2088,18 @@
   </si>
   <si>
     <t>Assumption: membership check plus one put. Fan-out uses the pub/sub topic, not a data store lookup (ADR-005).</t>
+  </si>
+  <si>
+    <t>User identity (Google subject, display name) is copied from the Google ID token at sign-in. Email is read from the token and not stored.</t>
+  </si>
+  <si>
+    <t>Personal data: Google subject, display name. Message text is user content. Classified external; no explicit payment, health, or regulated data requested by product.</t>
+  </si>
+  <si>
+    <t>Only Google subject and display name are held</t>
+  </si>
+  <si>
+    <t>pondId, duckId, googleSubject, displayName (unique per pond), createdAt</t>
   </si>
 </sst>
 </file>
@@ -4574,7 +4586,7 @@
         <v>142</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>453</v>
+        <v>681</v>
       </c>
       <c r="C27" s="2"/>
     </row>
@@ -4592,7 +4604,7 @@
         <v>144</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>455</v>
+        <v>682</v>
       </c>
       <c r="C29" s="2"/>
     </row>
@@ -5103,7 +5115,7 @@
         <v>505</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>512</v>
+        <v>683</v>
       </c>
       <c r="E31" s="2" t="s">
         <v>348</v>
@@ -5492,7 +5504,7 @@
         <v>553</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>554</v>
+        <v>684</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>555</v>

</xml_diff>

<commit_message>
finished phase 2 design: operational design, dependency and scope ADRs, decision log
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KMRvn11hi5T5syWSW5gyYX
</commit_message>
<xml_diff>
--- a/docs/discovery/Design Playbook - Quack.xlsx
+++ b/docs/discovery/Design Playbook - Quack.xlsx
@@ -7013,32 +7013,112 @@
       </c>
     </row>
     <row r="12" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="2"/>
-      <c r="B12" s="2"/>
-      <c r="C12" s="2"/>
-      <c r="D12" s="2"/>
-      <c r="E12" s="2"/>
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>DL-09</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Data store</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Aurora PostgreSQL Serverless v2; one table per entity; row-level security for pond and membership</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>docs/adr/adr-009-data-store.md</t>
+        </is>
+      </c>
     </row>
     <row r="13" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="2"/>
-      <c r="B13" s="2"/>
-      <c r="C13" s="2"/>
-      <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>DL-10</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Identity provider</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Google Sign-In, OpenID Connect ID token; no hosted user pool</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>docs/adr/adr-010-identity-provider.md</t>
+        </is>
+      </c>
     </row>
     <row r="14" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="2"/>
-      <c r="B14" s="2"/>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>DL-11</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Initial runtime dependencies</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>drizzle-orm and drizzle-kit, pg, iovalkey, jose, fastify, zod, ws, React with Vite</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>docs/adr/adr-011-initial-runtime-dependencies.md</t>
+        </is>
+      </c>
     </row>
     <row r="15" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="2"/>
-      <c r="B15" s="2"/>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>DL-12</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>MVP scope cuts</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>OOS-01 to OOS-11 and hosted user pools out of scope; each row names what adding it changes</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>docs/adr/adr-012-mvp-scope-cuts.md</t>
+        </is>
+      </c>
     </row>
     <row r="16" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="2"/>

</xml_diff>